<commit_message>
Updated logic to keep player selection the same between waves if player is still available (regardless if still in ovr range), redid table reference selection to coexist with madden weekly sim that reorders ContractOffer[] values
</commit_message>
<xml_diff>
--- a/Files/Madden26/IE/Season2/FreeAgency/Output/PlayerContract.xlsx
+++ b/Files/Madden26/IE/Season2/FreeAgency/Output/PlayerContract.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,17 +429,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SalaryTable</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>BonusTable</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Length</t>
         </is>
@@ -463,7 +475,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -480,7 +492,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -497,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -548,7 +560,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -565,7 +577,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -599,7 +611,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -616,7 +628,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -633,7 +645,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -650,7 +662,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -667,7 +679,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -684,7 +696,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -701,7 +713,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -718,7 +730,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -735,7 +747,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -752,7 +764,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -769,7 +781,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -820,7 +832,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -837,7 +849,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -854,7 +866,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -871,7 +883,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -888,7 +900,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -905,7 +917,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -922,7 +934,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -990,7 +1002,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1019,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1036,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1053,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1070,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1087,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1155,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1172,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1189,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1206,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1240,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1257,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1274,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1291,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1308,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1325,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1342,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1359,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1376,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1393,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1427,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1444,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1478,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1495,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1512,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1529,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1546,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1563,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1597,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1614,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1631,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1682,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1699,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1716,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1750,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1784,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1801,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1818,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1835,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1852,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1886,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1903,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1920,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1937,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1954,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1971,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1988,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1993,7 +2005,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2039,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2056,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2073,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2090,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2141,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2192,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2209,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2226,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2243,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2260,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2277,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2294,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2311,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2328,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2345,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2362,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2379,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2396,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2413,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2430,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2464,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2481,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2515,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2549,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2566,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2600,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2617,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2634,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2651,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2668,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2685,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2702,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2736,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2770,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2787,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2804,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2838,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2872,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2906,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2940,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2974,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2991,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -2996,7 +3008,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3042,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3093,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3110,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3127,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3144,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3178,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3195,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3200,7 +3212,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3229,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3234,7 +3246,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3263,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3280,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3297,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3314,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3331,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3348,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3365,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3382,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3399,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3416,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3433,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3450,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3467,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -3489,53 +3501,53 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>00000000000000000000000010110011</t>
+          <t>00101011010011100000000101101000</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101101001</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>00000000000000000000000010100000</t>
+          <t>00101011010011100000000101101010</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101101011</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>00000000000000000000000011110000</t>
+          <t>00101011010011100000000101101100</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101101101</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -3547,46 +3559,46 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>00000000000000000000000010110110</t>
+          <t>00101011010011100000000101101110</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101101111</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>00000000000000000000000011000111</t>
+          <t>00101011010011100000000101110000</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101110001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>00000000000000000000000011100100</t>
+          <t>00101011010011100000000101110010</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101110011</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -3598,29 +3610,29 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>00000000000000000000000010111001</t>
+          <t>00101011010011100000000101110100</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101110101</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>00000000000000000000000010011101</t>
+          <t>00101011010011100000000101110110</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101110111</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -3632,29 +3644,29 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>00000000000000000000000010011110</t>
+          <t>00101011010011100000000101111000</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101111001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>00000000000000000000000010110000</t>
+          <t>00101011010011100000000101111010</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101111011</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -3666,46 +3678,46 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>00000000000000000000000011010111</t>
+          <t>00101011010011100000000101111100</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101111101</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>00000000000000000000000010011111</t>
+          <t>00101011010011100000000101111110</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000101111111</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>00000000000000000000000001101101</t>
+          <t>00101011010011100000000110000000</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110000001</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -3717,29 +3729,29 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>00000000000000000000000011010100</t>
+          <t>00101011010011100000000110000010</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110000011</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>00000000000000000000000011100111</t>
+          <t>00101011010011100000000110000100</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110000101</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -3751,63 +3763,63 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>00000000000000000000000001001000</t>
+          <t>00101011010011100000000110000110</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110000111</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>00000000000000000000000010101010</t>
+          <t>00101011010011100000000110001000</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110001001</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>00000000000000000000000010101110</t>
+          <t>00101011010011100000000110001010</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110001011</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>00000000000000000000000010100100</t>
+          <t>00101011010011100000000110001100</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110001101</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -3819,46 +3831,46 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>00000000000000000000000010100011</t>
+          <t>00101011010011100000000110001110</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110001111</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>00000000000000000000000000100001</t>
+          <t>00101011010011100000000110010000</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110010001</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>00000000000000000000000010000000</t>
+          <t>00101011010011100000000110010010</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110010011</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -3870,12 +3882,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>00000000000000000000000011001110</t>
+          <t>00101011010011100000000110010100</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110010101</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -3887,12 +3899,12 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>00000000000000000000000010100111</t>
+          <t>00101011010011100000000110010110</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110010111</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -3904,46 +3916,46 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>00000000000000000000000011011101</t>
+          <t>00101011010011100000000110011000</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110011001</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>00000000000000000000000010010110</t>
+          <t>00101011010011100000000110011010</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110011011</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>00000000000000000000000010001111</t>
+          <t>00101011010011100000000110011100</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110011101</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -3955,29 +3967,29 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>00000000000000000000000010000100</t>
+          <t>00101011010011100000000110011110</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110011111</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>00000000000000000000000011100010</t>
+          <t>00101011010011100000000110100000</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110100001</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -3989,12 +4001,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>00000000000000000000000000100010</t>
+          <t>00101011010011100000000110100010</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110100011</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -4006,12 +4018,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>00000000000000000000000001011110</t>
+          <t>00101011010011100000000110100100</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110100101</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -4023,12 +4035,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>00000000000000000000000010111100</t>
+          <t>00101011010011100000000110100110</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110100111</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -4040,29 +4052,29 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>00000000000000000000000010011100</t>
+          <t>00101011010011100000000110101000</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110101001</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>00000000000000000000000001111011</t>
+          <t>00101011010011100000000110101010</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110101011</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -4074,63 +4086,63 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>00000000000000000000000001100100</t>
+          <t>00101011010011100000000110101100</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110101101</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>00000000000000000000000000101111</t>
+          <t>00101011010011100000000110101110</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110101111</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>00000000000000000000000011011011</t>
+          <t>00101011010011100000000110110000</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110110001</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>00000000000000000000000001000111</t>
+          <t>00101011010011100000000110110010</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110110011</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -4142,29 +4154,29 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>00000000000000000000000000011101</t>
+          <t>00101011010011100000000110110100</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110110101</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>00000000000000000000000011101110</t>
+          <t>00101011010011100000000110110110</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110110111</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -4176,97 +4188,97 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>00000000000000000000000010111101</t>
+          <t>00101011010011100000000110111000</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110111001</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>00000000000000000000000010101001</t>
+          <t>00101011010011100000000110111010</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110111011</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>00000000000000000000000010011000</t>
+          <t>00101011010011100000000110111100</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110111101</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>00000000000000000000000010101111</t>
+          <t>00101011010011100000000110111110</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000110111111</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>00000000000000000000000011000010</t>
+          <t>00101011010011100000000111000000</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111000001</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>00000000000000000000000011000110</t>
+          <t>00101011010011100000000111000010</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111000011</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -4278,12 +4290,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>00000000000000000000000011001000</t>
+          <t>00101011010011100000000111000100</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111000101</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -4295,29 +4307,29 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>00000000000000000000000010100010</t>
+          <t>00101011010011100000000111000110</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111000111</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>00000000000000000000000010110111</t>
+          <t>00101011010011100000000111001000</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111001001</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -4329,29 +4341,29 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>00000000000000000000000011001100</t>
+          <t>00101011010011100000000111001010</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111001011</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000011</t>
+          <t>00101011010011100000000111001100</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111001101</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -4363,29 +4375,29 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>00000000000000000000000000100111</t>
+          <t>00101011010011100000000111001110</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111001111</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>00000000000000000000000011001010</t>
+          <t>00101011010011100000000111010000</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111010001</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -4397,12 +4409,12 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>00000000000000000000000011101011</t>
+          <t>00101011010011100000000111010010</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111010011</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -4414,12 +4426,12 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>00000000000000000000000000011111</t>
+          <t>00101011010011100000000111010100</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111010101</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -4431,29 +4443,29 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111010110</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111010111</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>00000000000000000000000000011001</t>
+          <t>00101011010011100000000111011000</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111011001</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -4465,12 +4477,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>00000000000000000000000001100000</t>
+          <t>00101011010011100000000111011010</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111011011</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -4482,12 +4494,12 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>00000000000000000000000011100101</t>
+          <t>00101011010011100000000111011100</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111011101</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -4499,29 +4511,29 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>00000000000000000000000001000100</t>
+          <t>00101011010011100000000111011110</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111011111</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>00000000000000000000000010110100</t>
+          <t>00101011010011100000000111100000</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111100001</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -4533,29 +4545,29 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>00000000000000000000000011101001</t>
+          <t>00101011010011100000000111100010</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111100011</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>00000000000000000000000010001010</t>
+          <t>00101011010011100000000111100100</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111100101</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -4567,97 +4579,97 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>00000000000000000000000011010000</t>
+          <t>00101011010011100000000111100110</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111100111</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>00000000000000000000000001011001</t>
+          <t>00101011010011100000000111101000</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111101001</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>00000000000000000000000010010000</t>
+          <t>00101011010011100000000111101010</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111101011</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>00000000000000000000000001011000</t>
+          <t>00101011010011100000000111101100</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111101101</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>00000000000000000000000000001100</t>
+          <t>00101011010011100000000111101110</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111101111</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>00000000000000000000000011110111</t>
+          <t>00101011010011100000000111110000</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111110001</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -4669,12 +4681,12 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111011</t>
+          <t>00101011010011100000000111110010</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111110011</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -4686,97 +4698,97 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111001</t>
+          <t>00101011010011100000000111110100</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111110101</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111000</t>
+          <t>00101011010011100000000111110110</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111110111</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111010</t>
+          <t>00101011010011100000000111111000</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111111001</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111100</t>
+          <t>00101011010011100000000111111010</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111111011</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111111</t>
+          <t>00101011010011100000000111111100</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111111101</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111101</t>
+          <t>00101011010011100000000111111110</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000000111111111</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -4788,29 +4800,29 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>00000000000000000000000100000001</t>
+          <t>00101011010011100000001000000000</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000000001</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>00000000000000000000000011111110</t>
+          <t>00101011010011100000001000000010</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000000011</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -4822,969 +4834,969 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>00000000000000000000000100000100</t>
+          <t>00101011010011100000001000000100</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000000101</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>00000000000000000000000100000010</t>
+          <t>00101011010011100000001000000110</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000000111</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>00000000000000000000000100000000</t>
+          <t>00101011010011100000001000001000</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000001001</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>00000000000000000000000100000011</t>
+          <t>00101011010011100000001000001010</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000001011</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>00000000000000000000000100000111</t>
+          <t>00101011010011100000011111001011</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000011111001010</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>00000000000000000000000100000101</t>
+          <t>00101011010011100000011111001101</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000011111001100</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>00000000000000000000000010110101</t>
+          <t>00101011010011100000001000001100</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000001101</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>00000000000000000000000100001011</t>
+          <t>00101011010011100000001000001110</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000001111</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>00000000000000000000000100001011</t>
+          <t>00101011010011100000001000010000</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000010001</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>00000000000000000000000100001100</t>
+          <t>00101011010011100000001000010010</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000010011</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>00000000000000000000000100001101</t>
+          <t>00101011010011100000001000010100</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000010101</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>00000000000000000000000100001110</t>
+          <t>00101011010011100000001000010110</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000010111</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>00000000000000000000000100001111</t>
+          <t>00101011010011100000001000011000</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000011001</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010000</t>
+          <t>00101011010011100000001000011010</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000011011</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010001</t>
+          <t>00101011010011100000001000011100</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000011101</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010010</t>
+          <t>00101011010011100000001000011110</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000011111</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010011</t>
+          <t>00101011010011100000001000100000</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000100001</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010100</t>
+          <t>00101011010011100000001000100010</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000100011</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010101</t>
+          <t>00101011010011100000001000100100</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000100101</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010110</t>
+          <t>00101011010011100000001000100110</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000100111</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>00000000000000000000000100010111</t>
+          <t>00101011010011100000001000101000</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000101001</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011000</t>
+          <t>00101011010011100000001000101010</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000101011</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011001</t>
+          <t>00101011010011100000001000101100</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000101101</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011010</t>
+          <t>00101011010011100000001000101110</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000101111</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011011</t>
+          <t>00101011010011100000001000110000</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000110001</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011100</t>
+          <t>00101011010011100000001000110010</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000110011</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011101</t>
+          <t>00101011010011100000001000110100</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000110101</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011110</t>
+          <t>00101011010011100000001000110110</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000110111</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>00000000000000000000000100011111</t>
+          <t>00101011010011100000001000111000</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000111001</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100000</t>
+          <t>00101011010011100000001000111010</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000111011</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100001</t>
+          <t>00101011010011100000001000111100</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000111101</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100010</t>
+          <t>00101011010011100000001000111110</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001000111111</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100011</t>
+          <t>00101011010011100000001001000000</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001000001</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100100</t>
+          <t>00101011010011100000001001000010</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001000011</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100101</t>
+          <t>00101011010011100000001001000100</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001000101</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100110</t>
+          <t>00101011010011100000001001000110</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001000111</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>00000000000000000000000100100111</t>
+          <t>00101011010011100000001001001000</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001001001</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101000</t>
+          <t>00101011010011100000001001001010</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001001011</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101001</t>
+          <t>00101011010011100000001001001100</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001001101</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101010</t>
+          <t>00101011010011100000001001001110</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001001111</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101011</t>
+          <t>00101011010011100000011111000111</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000011111000110</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101100</t>
+          <t>00101011010011100000011111000101</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000011111000100</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101101</t>
+          <t>00101011010011100000001001010000</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001010001</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101110</t>
+          <t>00101011010011100000001001010010</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001010011</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>00000000000000000000000100101111</t>
+          <t>00101011010011100000001001010100</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001010101</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110000</t>
+          <t>00101011010011100000001001010110</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001010111</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110001</t>
+          <t>00101011010011100000001001011000</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001011001</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110010</t>
+          <t>00101011010011100000001001011010</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001011011</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110011</t>
+          <t>00101011010011100000001001011100</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001011101</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110100</t>
+          <t>00101011010011100000001001011110</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001011111</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110101</t>
+          <t>00101011010011100000001001100000</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001100001</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110110</t>
+          <t>00101011010011100000001001100010</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001100011</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>00000000000000000000000100110111</t>
+          <t>00101011010011100000001001100100</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001100101</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>00000000000000000000000100111000</t>
+          <t>00101011010011100000001001100110</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001100111</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>00000000000000000000000100111001</t>
+          <t>00101011010011100000001001101000</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001101001</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>00000000000000000000000100111010</t>
+          <t>00101011010011100000001001101010</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001101011</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>00000000000000000000000100111011</t>
+          <t>00101011010011100000001001101100</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>00000000000000000000000000000000</t>
+          <t>00101011010011100000001001101101</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>